<commit_message>
Retire l'article de test de packing_liste.xlsx (fichier de travail réel)
</commit_message>
<xml_diff>
--- a/packing_liste.xlsx
+++ b/packing_liste.xlsx
@@ -48781,172 +48781,160 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>05449000243195</t>
+          <t>13179142040244</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>TEST — Coca-Cola 33cl (EAN-13)</t>
+          <t>BTE150G FRUIT ASSORTX012-VA</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>TEST001</t>
+          <t>901601698</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>13179142040244</t>
+          <t>13179142040251</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>BTE150G FRUIT ASSORTX012-VA</t>
+          <t>BTE150G MACEDOINE X012-VA</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>901601698</t>
+          <t>901601699</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>13179142040251</t>
+          <t>13179142040299</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>BTE150G MACEDOINE X012-VA</t>
+          <t>BTE100G LAMELLE ORANGX12-VA</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>901601699</t>
+          <t>901602259</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>13179142040299</t>
+          <t>13179142040305</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>BTE100G LAMELLE ORANGX12-VA</t>
+          <t>BTE150G BIGARREAUX X012-VA</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>901602259</t>
+          <t>901602260</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>13179142040305</t>
+          <t>03179143054458</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>BTE150G BIGARREAUX X012-VA</t>
+          <t>BLISTER COLORANTS LIQUIDES VAHINE Espagne Portugal</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>901602260</t>
+          <t>804880</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>03179143054458</t>
+          <t>03179143054441</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>BLISTER COLORANTS LIQUIDES VAHINE Espagne Portugal</t>
+          <t>BLISTER COLORANTS LIQUIDES VAHINE Belgique</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>804880</t>
+          <t>802410</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>03179143054441</t>
+          <t>13179140633455</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>BLISTER COLORANTS LIQUIDES VAHINE Belgique</t>
+          <t>BLISTER COLORANTS LIQUIDES VAHINE France</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>802410</t>
+          <t>202330</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>13179140633455</t>
+          <t>00327592305246</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>BLISTER COLORANTS LIQUIDES VAHINE France</t>
+          <t>BLIS.COLORANT PATIS. GR x12-VAHINE</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>202330</t>
+          <t>M010153</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>00327592305246</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>BLIS.COLORANT PATIS. GR x12-VAHINE</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>M010153</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
           <t>13179142066589</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>PAV 20S SUCRE VANILLEX11-VA</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>901770216</t>
         </is>
       </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>

</xml_diff>